<commit_message>
Update self_reported_results.xlsx with latest data revisions
</commit_message>
<xml_diff>
--- a/static/data/self_reported_results.xlsx
+++ b/static/data/self_reported_results.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="730" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="296">
   <si>
     <t>Model</t>
   </si>
@@ -894,6 +894,30 @@
   </si>
   <si>
     <t>https://drive.google.com/file/d/1FP7U6QlGn1NUqQucLnUzKy_IfKotYQb1/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>Turix (computer_13, 50 steps)</t>
+  </si>
+  <si>
+    <t>New Generation Technology</t>
+  </si>
+  <si>
+    <t>https://github.com/xlang-ai/OSWorld</t>
+  </si>
+  <si>
+    <t>Pei et al., '26</t>
+  </si>
+  <si>
+    <t>Provider: vmware, Obs: screenshot, Action: computer_13, Max steps: 50, Parallel envs: 3, Commit: 3afe772dc54e5c47ef6916f0de27f7c2b5c34d2b, Testset: evaluation_examples/test_nogdrive_turix.json</t>
+  </si>
+  <si>
+    <t>self_report_osworld_turix_2026-03-23.zip</t>
+  </si>
+  <si>
+    <t>Mar 23, 2026</t>
+  </si>
+  <si>
+    <t>Provider: VMware; Observation type: screenshot; Action space: computer_13; Max steps: 50; Parallel environments: 3; Run date: 2026-03-23; Repository: xlang-ai/OSWorld (fork); Commit: 3afe772dc54e5c47ef6916f0de27f7c2b5c34d2b; Test set: evaluation_examples/test_nogdrive_turix.json (no Google Drive).</t>
   </si>
 </sst>
 </file>
@@ -1834,9 +1858,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr/>
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:J57"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
@@ -1901,229 +1925,228 @@
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>288</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>17</v>
+        <v>289</v>
+      </c>
+      <c r="C3" t="s" s="2">
+        <v>290</v>
       </c>
       <c r="D3" t="s">
-        <v>18</v>
+        <v>291</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3" s="5">
-        <v>45.2</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>20</v>
+        <v>295</v>
+      </c>
+      <c r="F3" t="s">
+        <v>293</v>
+      </c>
+      <c r="G3">
+        <v>57.99</v>
+      </c>
+      <c r="H3" t="s" s="1">
+        <v>294</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>23</v>
+        <v>16</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="D4" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="E4" t="s">
         <v>13</v>
       </c>
-      <c r="F4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4">
-        <v>42.9</v>
+      <c r="F4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" s="5">
+        <v>45.2</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>28</v>
+        <v>22</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>23</v>
       </c>
       <c r="D5" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E5" t="s">
-        <v>30</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>31</v>
+        <v>13</v>
+      </c>
+      <c r="F5" t="s">
+        <v>13</v>
       </c>
       <c r="G5">
-        <v>42.5</v>
+        <v>42.9</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="D6" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="E6" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>37</v>
+        <v>30</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="G6">
-        <v>41.4</v>
+        <v>42.5</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="I6" s="6"/>
+        <v>32</v>
+      </c>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7" t="s">
-        <v>40</v>
+        <v>34</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="E7" t="s">
         <v>13</v>
       </c>
-      <c r="F7" t="s">
-        <v>13</v>
+      <c r="F7" s="3" t="s">
+        <v>37</v>
       </c>
       <c r="G7">
-        <v>38.1</v>
+        <v>41.4</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="I7" s="6"/>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>44</v>
+        <v>22</v>
+      </c>
+      <c r="C8" t="s">
+        <v>40</v>
       </c>
       <c r="D8" t="s">
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="E8" t="s">
-        <v>46</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>47</v>
+        <v>13</v>
+      </c>
+      <c r="F8" t="s">
+        <v>13</v>
       </c>
       <c r="G8">
-        <v>35.27</v>
+        <v>38.1</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="I8" s="6"/>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" t="s">
-        <v>50</v>
+        <v>43</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>44</v>
       </c>
       <c r="D9" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="E9" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="G9">
-        <v>34.5</v>
+        <v>35.27</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="I9" s="6"/>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B10" t="s">
-        <v>53</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>54</v>
+        <v>34</v>
+      </c>
+      <c r="C10" t="s">
+        <v>50</v>
       </c>
       <c r="D10" t="s">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="E10" t="s">
         <v>13</v>
       </c>
-      <c r="F10" t="s">
-        <v>13</v>
+      <c r="F10" s="3" t="s">
+        <v>37</v>
       </c>
       <c r="G10">
-        <v>29.9</v>
+        <v>34.5</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="I10" s="6"/>
     </row>
     <row r="11" spans="1:9">
       <c r="A11" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B11" t="s">
-        <v>58</v>
-      </c>
-      <c r="C11" t="s">
-        <v>59</v>
+        <v>53</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>54</v>
       </c>
       <c r="D11" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="E11" t="s">
         <v>13</v>
@@ -2131,242 +2154,242 @@
       <c r="F11" t="s">
         <v>13</v>
       </c>
-      <c r="G11" t="s">
-        <v>61</v>
+      <c r="G11">
+        <v>29.9</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="I11" s="6"/>
     </row>
     <row r="12" spans="1:9">
       <c r="A12" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="B12" t="s">
-        <v>64</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>65</v>
+        <v>58</v>
+      </c>
+      <c r="C12" t="s">
+        <v>59</v>
       </c>
       <c r="D12" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="E12" t="s">
-        <v>67</v>
+        <v>13</v>
       </c>
       <c r="F12" t="s">
         <v>13</v>
       </c>
-      <c r="G12">
-        <v>27.04</v>
+      <c r="G12" t="s">
+        <v>61</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="I12" s="6"/>
     </row>
     <row r="13" spans="1:9">
       <c r="A13" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="B13" t="s">
-        <v>34</v>
-      </c>
-      <c r="C13" t="s">
-        <v>50</v>
+        <v>64</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>65</v>
       </c>
       <c r="D13" t="s">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="E13" t="s">
-        <v>13</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>37</v>
+        <v>67</v>
+      </c>
+      <c r="F13" t="s">
+        <v>13</v>
       </c>
       <c r="G13">
-        <v>27</v>
+        <v>27.04</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>51</v>
+        <v>68</v>
       </c>
       <c r="I13" s="6"/>
     </row>
     <row r="14" spans="1:9">
       <c r="A14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" t="s">
+        <v>50</v>
+      </c>
+      <c r="D14" t="s">
+        <v>36</v>
+      </c>
+      <c r="E14" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G14">
         <v>27</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D14" t="s">
-        <v>29</v>
-      </c>
-      <c r="E14" t="s">
-        <v>13</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="G14">
-        <v>26.92</v>
-      </c>
       <c r="H14" s="1" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="I14" s="6"/>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B15" t="s">
-        <v>58</v>
-      </c>
-      <c r="C15" t="s">
-        <v>59</v>
+        <v>27</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="D15" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="E15" t="s">
         <v>13</v>
       </c>
-      <c r="F15" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" t="s">
-        <v>73</v>
+      <c r="F15" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G15">
+        <v>26.92</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>62</v>
+        <v>32</v>
       </c>
       <c r="I15" s="6"/>
     </row>
     <row r="16" spans="1:9">
       <c r="A16" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B16" t="s">
-        <v>64</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>65</v>
+        <v>58</v>
+      </c>
+      <c r="C16" t="s">
+        <v>59</v>
       </c>
       <c r="D16" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="E16" t="s">
-        <v>75</v>
+        <v>13</v>
       </c>
       <c r="F16" t="s">
         <v>13</v>
       </c>
-      <c r="G16">
-        <v>25.02</v>
+      <c r="G16" t="s">
+        <v>73</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="I16" s="6"/>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B17" t="s">
-        <v>27</v>
-      </c>
-      <c r="C17" t="s">
-        <v>77</v>
+        <v>64</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>65</v>
       </c>
       <c r="D17" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="E17" t="s">
-        <v>13</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>79</v>
+        <v>75</v>
+      </c>
+      <c r="F17" t="s">
+        <v>13</v>
       </c>
       <c r="G17">
-        <v>24.6</v>
+        <v>25.02</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="I17" s="6"/>
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="B18" t="s">
-        <v>64</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>65</v>
+        <v>27</v>
+      </c>
+      <c r="C18" t="s">
+        <v>77</v>
       </c>
       <c r="D18" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="E18" t="s">
-        <v>82</v>
-      </c>
-      <c r="F18" t="s">
-        <v>13</v>
+        <v>13</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>79</v>
       </c>
       <c r="G18">
-        <v>22.74</v>
+        <v>24.6</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="I18" s="6"/>
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B19" t="s">
-        <v>27</v>
-      </c>
-      <c r="C19" t="s">
-        <v>77</v>
+        <v>64</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>65</v>
       </c>
       <c r="D19" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="E19" t="s">
-        <v>13</v>
+        <v>82</v>
       </c>
       <c r="F19" t="s">
         <v>13</v>
       </c>
       <c r="G19">
-        <v>22.7</v>
+        <v>22.74</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="I19" s="6"/>
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B20" t="s">
-        <v>58</v>
+        <v>27</v>
       </c>
       <c r="C20" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="D20" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="E20" t="s">
         <v>13</v>
@@ -2375,79 +2398,79 @@
         <v>13</v>
       </c>
       <c r="G20">
-        <v>22</v>
+        <v>22.7</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="I20" s="6"/>
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B21" t="s">
-        <v>64</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>65</v>
+        <v>58</v>
+      </c>
+      <c r="C21" t="s">
+        <v>85</v>
       </c>
       <c r="D21" t="s">
-        <v>66</v>
+        <v>86</v>
       </c>
       <c r="E21" t="s">
-        <v>89</v>
+        <v>13</v>
       </c>
       <c r="F21" t="s">
         <v>13</v>
       </c>
       <c r="G21">
-        <v>21.8</v>
+        <v>22</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
       <c r="I21" s="6"/>
     </row>
     <row r="22" spans="1:9">
       <c r="A22" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B22" t="s">
-        <v>58</v>
-      </c>
-      <c r="C22" t="s">
-        <v>59</v>
+        <v>64</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>65</v>
       </c>
       <c r="D22" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="E22" t="s">
-        <v>13</v>
+        <v>89</v>
       </c>
       <c r="F22" t="s">
         <v>13</v>
       </c>
-      <c r="G22" t="s">
-        <v>91</v>
+      <c r="G22">
+        <v>21.8</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="I22" s="6"/>
     </row>
     <row r="23" spans="1:9">
       <c r="A23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B23" t="s">
-        <v>93</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>94</v>
+        <v>58</v>
+      </c>
+      <c r="C23" t="s">
+        <v>59</v>
       </c>
       <c r="D23" t="s">
-        <v>18</v>
+        <v>60</v>
       </c>
       <c r="E23" t="s">
         <v>13</v>
@@ -2455,26 +2478,26 @@
       <c r="F23" t="s">
         <v>13</v>
       </c>
-      <c r="G23">
-        <v>20.2</v>
+      <c r="G23" t="s">
+        <v>91</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>95</v>
+        <v>62</v>
       </c>
       <c r="I23" s="6"/>
     </row>
     <row r="24" spans="1:9">
       <c r="A24" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B24" t="s">
-        <v>22</v>
-      </c>
-      <c r="C24" t="s">
-        <v>40</v>
+        <v>93</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>94</v>
       </c>
       <c r="D24" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="E24" t="s">
         <v>13</v>
@@ -2483,25 +2506,25 @@
         <v>13</v>
       </c>
       <c r="G24">
-        <v>19.7</v>
+        <v>20.2</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>41</v>
+        <v>95</v>
       </c>
       <c r="I24" s="6"/>
     </row>
     <row r="25" spans="1:9">
       <c r="A25" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B25" t="s">
-        <v>58</v>
+        <v>22</v>
       </c>
       <c r="C25" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="D25" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="E25" t="s">
         <v>13</v>
@@ -2509,26 +2532,26 @@
       <c r="F25" t="s">
         <v>13</v>
       </c>
-      <c r="G25" t="s">
-        <v>98</v>
+      <c r="G25">
+        <v>19.7</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>62</v>
+        <v>41</v>
       </c>
       <c r="I25" s="6"/>
     </row>
     <row r="26" spans="1:9">
       <c r="A26" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B26" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="C26" t="s">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="D26" t="s">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="E26" t="s">
         <v>13</v>
@@ -2536,17 +2559,17 @@
       <c r="F26" t="s">
         <v>13</v>
       </c>
-      <c r="G26">
-        <v>18.8</v>
+      <c r="G26" t="s">
+        <v>98</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="I26" s="6"/>
     </row>
     <row r="27" spans="1:9">
       <c r="A27" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B27" t="s">
         <v>27</v>
@@ -2564,7 +2587,7 @@
         <v>13</v>
       </c>
       <c r="G27">
-        <v>18.7</v>
+        <v>18.8</v>
       </c>
       <c r="H27" s="1" t="s">
         <v>80</v>
@@ -2573,7 +2596,7 @@
     </row>
     <row r="28" spans="1:9">
       <c r="A28" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B28" t="s">
         <v>27</v>
@@ -2591,7 +2614,7 @@
         <v>13</v>
       </c>
       <c r="G28">
-        <v>17.7</v>
+        <v>18.7</v>
       </c>
       <c r="H28" s="1" t="s">
         <v>80</v>
@@ -2600,16 +2623,16 @@
     </row>
     <row r="29" spans="1:9">
       <c r="A29" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B29" t="s">
-        <v>64</v>
+        <v>27</v>
       </c>
       <c r="C29" t="s">
-        <v>103</v>
+        <v>77</v>
       </c>
       <c r="D29" t="s">
-        <v>104</v>
+        <v>78</v>
       </c>
       <c r="E29" t="s">
         <v>13</v>
@@ -2618,25 +2641,25 @@
         <v>13</v>
       </c>
       <c r="G29">
-        <v>17.04</v>
+        <v>17.7</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="I29" s="6"/>
     </row>
     <row r="30" spans="1:9">
       <c r="A30" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B30" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="C30" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
       <c r="D30" t="s">
-        <v>60</v>
+        <v>104</v>
       </c>
       <c r="E30" t="s">
         <v>13</v>
@@ -2644,26 +2667,26 @@
       <c r="F30" t="s">
         <v>13</v>
       </c>
-      <c r="G30" t="s">
-        <v>107</v>
+      <c r="G30">
+        <v>17.04</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>62</v>
+        <v>105</v>
       </c>
       <c r="I30" s="6"/>
     </row>
     <row r="31" spans="1:9">
       <c r="A31" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B31" t="s">
-        <v>109</v>
+        <v>58</v>
       </c>
       <c r="C31" t="s">
-        <v>110</v>
+        <v>59</v>
       </c>
       <c r="D31" t="s">
-        <v>111</v>
+        <v>60</v>
       </c>
       <c r="E31" t="s">
         <v>13</v>
@@ -2671,53 +2694,53 @@
       <c r="F31" t="s">
         <v>13</v>
       </c>
-      <c r="G31">
-        <v>15.15</v>
+      <c r="G31" t="s">
+        <v>107</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>112</v>
+        <v>62</v>
       </c>
       <c r="I31" s="6"/>
     </row>
     <row r="32" spans="1:9">
       <c r="A32" t="s">
+        <v>108</v>
+      </c>
+      <c r="B32" t="s">
+        <v>109</v>
+      </c>
+      <c r="C32" t="s">
+        <v>110</v>
+      </c>
+      <c r="D32" t="s">
+        <v>111</v>
+      </c>
+      <c r="E32" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32" t="s">
+        <v>13</v>
+      </c>
+      <c r="G32">
+        <v>15.15</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="I32" s="6"/>
+    </row>
+    <row r="33" spans="1:9">
+      <c r="A33" t="s">
         <v>113</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B33" t="s">
         <v>114</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C33" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D33" t="s">
         <v>116</v>
-      </c>
-      <c r="E32" t="s">
-        <v>13</v>
-      </c>
-      <c r="F32" t="s">
-        <v>13</v>
-      </c>
-      <c r="G32">
-        <v>14.9</v>
-      </c>
-      <c r="H32" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="I32" s="6"/>
-    </row>
-    <row r="33" spans="1:10">
-      <c r="A33" t="s">
-        <v>118</v>
-      </c>
-      <c r="B33" t="s">
-        <v>58</v>
-      </c>
-      <c r="C33" t="s">
-        <v>85</v>
-      </c>
-      <c r="D33" t="s">
-        <v>86</v>
       </c>
       <c r="E33" t="s">
         <v>13</v>
@@ -2729,22 +2752,22 @@
         <v>14.9</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>87</v>
+        <v>117</v>
       </c>
       <c r="I33" s="6"/>
     </row>
     <row r="34" spans="1:10">
       <c r="A34" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B34" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="C34" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="D34" t="s">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="E34" t="s">
         <v>13</v>
@@ -2753,25 +2776,25 @@
         <v>13</v>
       </c>
       <c r="G34">
-        <v>14.79</v>
+        <v>14.9</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>105</v>
+        <v>87</v>
       </c>
       <c r="I34" s="6"/>
     </row>
     <row r="35" spans="1:10">
       <c r="A35" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B35" t="s">
-        <v>93</v>
+        <v>64</v>
       </c>
       <c r="C35" t="s">
-        <v>121</v>
+        <v>103</v>
       </c>
       <c r="D35" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="E35" t="s">
         <v>13</v>
@@ -2780,16 +2803,16 @@
         <v>13</v>
       </c>
       <c r="G35">
-        <v>14.63</v>
+        <v>14.79</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>123</v>
+        <v>105</v>
       </c>
       <c r="I35" s="6"/>
     </row>
     <row r="36" spans="1:10">
       <c r="A36" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="B36" t="s">
         <v>93</v>
@@ -2807,7 +2830,7 @@
         <v>13</v>
       </c>
       <c r="G36">
-        <v>11.65</v>
+        <v>14.63</v>
       </c>
       <c r="H36" s="1" t="s">
         <v>123</v>
@@ -2816,16 +2839,16 @@
     </row>
     <row r="37" spans="1:10">
       <c r="A37" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B37" t="s">
-        <v>64</v>
+        <v>93</v>
       </c>
       <c r="C37" t="s">
-        <v>103</v>
+        <v>121</v>
       </c>
       <c r="D37" t="s">
-        <v>104</v>
+        <v>122</v>
       </c>
       <c r="E37" t="s">
         <v>13</v>
@@ -2834,25 +2857,25 @@
         <v>13</v>
       </c>
       <c r="G37">
-        <v>10.26</v>
+        <v>11.65</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>105</v>
+        <v>123</v>
       </c>
       <c r="I37" s="6"/>
     </row>
     <row r="38" spans="1:10">
       <c r="A38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B38" t="s">
-        <v>127</v>
+        <v>64</v>
       </c>
       <c r="C38" t="s">
-        <v>128</v>
+        <v>103</v>
       </c>
       <c r="D38" t="s">
-        <v>129</v>
+        <v>104</v>
       </c>
       <c r="E38" t="s">
         <v>13</v>
@@ -2861,79 +2884,79 @@
         <v>13</v>
       </c>
       <c r="G38">
-        <v>9.21</v>
+        <v>10.26</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="J38" s="6"/>
+        <v>105</v>
+      </c>
+      <c r="I38" s="6"/>
     </row>
     <row r="39" spans="1:10">
       <c r="A39" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B39" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C39" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="D39" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="E39" t="s">
-        <v>134</v>
+        <v>13</v>
       </c>
       <c r="F39" t="s">
         <v>13</v>
       </c>
       <c r="G39">
-        <v>8.8</v>
+        <v>9.21</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="I39" s="6"/>
+        <v>123</v>
+      </c>
+      <c r="J39" s="6"/>
     </row>
     <row r="40" spans="1:10">
       <c r="A40" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B40" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C40" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="D40" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="E40" t="s">
-        <v>13</v>
+        <v>134</v>
       </c>
       <c r="F40" t="s">
         <v>13</v>
       </c>
       <c r="G40">
-        <v>8.7</v>
+        <v>8.8</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="I40" s="6"/>
     </row>
     <row r="41" spans="1:10">
       <c r="A41" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="B41" t="s">
-        <v>142</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>143</v>
+        <v>137</v>
+      </c>
+      <c r="C41" t="s">
+        <v>138</v>
       </c>
       <c r="D41" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="E41" t="s">
         <v>13</v>
@@ -2942,238 +2965,238 @@
         <v>13</v>
       </c>
       <c r="G41">
-        <v>8.22</v>
+        <v>8.7</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="I41" s="6"/>
     </row>
     <row r="42" spans="1:10">
       <c r="A42" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B42" t="s">
-        <v>147</v>
-      </c>
-      <c r="C42" t="s">
-        <v>148</v>
+        <v>142</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>143</v>
       </c>
       <c r="D42" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E42" t="s">
-        <v>134</v>
+        <v>13</v>
       </c>
       <c r="F42" t="s">
         <v>13</v>
       </c>
       <c r="G42">
-        <v>8.12</v>
+        <v>8.22</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>112</v>
+        <v>145</v>
       </c>
       <c r="I42" s="6"/>
     </row>
     <row r="43" spans="1:10">
       <c r="A43" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B43" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C43" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="D43" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="E43" t="s">
         <v>134</v>
       </c>
-      <c r="F43" s="3" t="s">
-        <v>154</v>
+      <c r="F43" t="s">
+        <v>13</v>
       </c>
       <c r="G43">
-        <v>7.81</v>
+        <v>8.12</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="J43" s="6"/>
+        <v>112</v>
+      </c>
+      <c r="I43" s="6"/>
     </row>
     <row r="44" spans="1:10">
       <c r="A44" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="B44" t="s">
-        <v>22</v>
+        <v>151</v>
       </c>
       <c r="C44" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="D44" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="E44" t="s">
         <v>134</v>
       </c>
-      <c r="F44" s="2" t="s">
-        <v>159</v>
+      <c r="F44" s="3" t="s">
+        <v>154</v>
       </c>
       <c r="G44">
-        <v>7.69</v>
+        <v>7.81</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="I44" s="6"/>
+        <v>155</v>
+      </c>
+      <c r="J44" s="6"/>
     </row>
     <row r="45" spans="1:10">
       <c r="A45" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="B45" t="s">
-        <v>162</v>
+        <v>22</v>
       </c>
       <c r="C45" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="D45" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="E45" t="s">
         <v>134</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="G45">
-        <v>5.8</v>
+        <v>7.69</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="J45" s="6"/>
+        <v>160</v>
+      </c>
+      <c r="I45" s="6"/>
     </row>
     <row r="46" spans="1:10">
       <c r="A46" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="B46" t="s">
-        <v>22</v>
+        <v>162</v>
       </c>
       <c r="C46" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="D46" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="E46" t="s">
         <v>134</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="G46">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="I46" s="6"/>
+        <v>166</v>
+      </c>
+      <c r="J46" s="6"/>
     </row>
     <row r="47" spans="1:10">
       <c r="A47" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="B47" t="s">
-        <v>162</v>
+        <v>22</v>
       </c>
       <c r="C47" t="s">
-        <v>171</v>
+        <v>157</v>
       </c>
       <c r="D47" t="s">
-        <v>172</v>
+        <v>158</v>
       </c>
       <c r="E47" t="s">
         <v>134</v>
       </c>
-      <c r="F47" s="3" t="s">
-        <v>173</v>
+      <c r="F47" s="2" t="s">
+        <v>168</v>
       </c>
       <c r="G47">
         <v>5.4</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="I47" s="6"/>
     </row>
     <row r="48" spans="1:10">
       <c r="A48" t="s">
+        <v>170</v>
+      </c>
+      <c r="B48" t="s">
+        <v>162</v>
+      </c>
+      <c r="C48" t="s">
+        <v>171</v>
+      </c>
+      <c r="D48" t="s">
+        <v>172</v>
+      </c>
+      <c r="E48" t="s">
+        <v>134</v>
+      </c>
+      <c r="F48" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="G48">
+        <v>5.4</v>
+      </c>
+      <c r="H48" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="I48" s="6"/>
+    </row>
+    <row r="49" spans="1:10">
+      <c r="A49" t="s">
         <v>156</v>
-      </c>
-      <c r="B48" t="s">
-        <v>22</v>
-      </c>
-      <c r="C48" t="s">
-        <v>157</v>
-      </c>
-      <c r="D48" t="s">
-        <v>158</v>
-      </c>
-      <c r="E48" t="s">
-        <v>134</v>
-      </c>
-      <c r="F48" t="s">
-        <v>13</v>
-      </c>
-      <c r="G48">
-        <v>5.26</v>
-      </c>
-      <c r="H48" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="I48" s="6"/>
-    </row>
-    <row r="49" spans="1:9">
-      <c r="A49" t="s">
-        <v>175</v>
       </c>
       <c r="B49" t="s">
         <v>22</v>
       </c>
       <c r="C49" t="s">
-        <v>176</v>
+        <v>157</v>
       </c>
       <c r="D49" t="s">
-        <v>177</v>
+        <v>158</v>
       </c>
       <c r="E49" t="s">
         <v>134</v>
       </c>
-      <c r="F49" s="2" t="s">
-        <v>178</v>
+      <c r="F49" t="s">
+        <v>13</v>
       </c>
       <c r="G49">
-        <v>5.03</v>
+        <v>5.26</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>179</v>
+        <v>166</v>
       </c>
       <c r="I49" s="6"/>
     </row>
     <row r="50" spans="1:9">
       <c r="A50" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="B50" t="s">
         <v>22</v>
       </c>
       <c r="C50" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="D50" t="s">
         <v>177</v>
@@ -3182,37 +3205,37 @@
         <v>134</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="G50">
-        <v>3.77</v>
+        <v>5.03</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="I50" s="6"/>
     </row>
     <row r="51" spans="1:9">
       <c r="A51" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B51" t="s">
-        <v>185</v>
+        <v>22</v>
       </c>
       <c r="C51" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="D51" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
       <c r="E51" t="s">
         <v>134</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="G51">
-        <v>3.33</v>
+        <v>3.77</v>
       </c>
       <c r="H51" s="1" t="s">
         <v>183</v>
@@ -3221,174 +3244,201 @@
     </row>
     <row r="52" spans="1:9">
       <c r="A52" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="B52" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C52" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="D52" t="s">
-        <v>86</v>
+        <v>187</v>
       </c>
       <c r="E52" t="s">
         <v>134</v>
       </c>
-      <c r="F52" t="s">
-        <v>13</v>
+      <c r="F52" s="2" t="s">
+        <v>188</v>
       </c>
       <c r="G52">
-        <v>2.42</v>
+        <v>3.33</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>166</v>
+        <v>183</v>
       </c>
       <c r="I52" s="6"/>
     </row>
     <row r="53" spans="1:9">
       <c r="A53" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="B53" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C53" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="D53" t="s">
-        <v>195</v>
+        <v>86</v>
       </c>
       <c r="E53" t="s">
         <v>134</v>
       </c>
-      <c r="F53" s="2" t="s">
-        <v>196</v>
+      <c r="F53" t="s">
+        <v>13</v>
       </c>
       <c r="G53">
         <v>2.42</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="I53" s="6"/>
     </row>
     <row r="54" spans="1:9">
       <c r="A54" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="B54" t="s">
-        <v>131</v>
+        <v>193</v>
       </c>
       <c r="C54" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D54" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E54" t="s">
         <v>134</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="G54">
         <v>2.42</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>201</v>
+        <v>183</v>
       </c>
       <c r="I54" s="6"/>
     </row>
     <row r="55" spans="1:9">
       <c r="A55" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="B55" t="s">
-        <v>203</v>
+        <v>131</v>
       </c>
       <c r="C55" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="D55" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="E55" t="s">
         <v>134</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="G55">
-        <v>1.88</v>
+        <v>2.42</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>183</v>
-      </c>
+        <v>201</v>
+      </c>
+      <c r="I55" s="6"/>
     </row>
     <row r="56" spans="1:9">
       <c r="A56" t="s">
+        <v>202</v>
+      </c>
+      <c r="B56" t="s">
+        <v>203</v>
+      </c>
+      <c r="C56" t="s">
+        <v>194</v>
+      </c>
+      <c r="D56" t="s">
+        <v>204</v>
+      </c>
+      <c r="E56" t="s">
+        <v>134</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="G56">
+        <v>1.88</v>
+      </c>
+      <c r="H56" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9">
+      <c r="A57" t="s">
         <v>206</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B57" t="s">
         <v>147</v>
       </c>
-      <c r="C56" s="4" t="s">
+      <c r="C57" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="D56" t="s">
+      <c r="D57" t="s">
         <v>208</v>
       </c>
-      <c r="E56" t="s">
-        <v>134</v>
-      </c>
-      <c r="F56" t="s">
-        <v>13</v>
-      </c>
-      <c r="G56">
+      <c r="E57" t="s">
+        <v>134</v>
+      </c>
+      <c r="F57" t="s">
+        <v>13</v>
+      </c>
+      <c r="G57">
         <v>1.11</v>
       </c>
-      <c r="H56" s="1" t="s">
+      <c r="H57" s="1" t="s">
         <v>166</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C41" r:id="rId1" display="https://arxiv.org/abs/2504.07491"/>
-    <hyperlink ref="C5" r:id="rId2" display="https://seed-tars.com/1.5"/>
-    <hyperlink ref="C6" r:id="rId3" display="https://github.com/simular-ai/Agent-S"/>
-    <hyperlink ref="C14" r:id="rId2" display="https://seed-tars.com/1.5" tooltip="https://seed-tars.com/1.5"/>
-    <hyperlink ref="F5" r:id="rId4" display="https://drive.google.com/file/d/1e7SCYqpxFX2FCGEOhf6jcVvwkx3leIKf/view?usp=drive_link"/>
-    <hyperlink ref="F17" r:id="rId5" display="https://drive.google.com/file/d/1vUWlXVenkOc5F1s-z8DdpfU4Y5fUMssr/view?usp=drive_link" tooltip="https://drive.google.com/file/d/1vUWlXVenkOc5F1s-z8DdpfU4Y5fUMssr/view?usp=drive_link"/>
-    <hyperlink ref="F43" r:id="rId6" display="https://drive.google.com/drive/folders/14_xlL-e0-0INq2O1THbhFKi6Z0bgfwR4?usp=drive_link"/>
-    <hyperlink ref="F47" r:id="rId7" display="https://drive.google.com/drive/folders/1j-YVzEGAGWxXgse75MCnhUCTVuejM76A?usp=drive_link"/>
-    <hyperlink ref="F9" r:id="rId8" display="https://drive.google.com/drive/folders/18PTnMwgyhxIWTVNLMwf0sbzhvh9AlVqE?usp=drive_link" tooltip="https://drive.google.com/drive/folders/18PTnMwgyhxIWTVNLMwf0sbzhvh9AlVqE?usp=drive_link"/>
-    <hyperlink ref="F46" r:id="rId9" display="https://drive.google.com/drive/folders/1NLsHdLUNZOHsEC5xNZ4e4PHkDC5IELjj?usp=drive_link"/>
-    <hyperlink ref="F54" r:id="rId10" display="https://drive.google.com/drive/folders/1iBOXZpknCi1Fqzg0fQMG6CZc9NWrwdkf?usp=drive_link"/>
-    <hyperlink ref="F45" r:id="rId11" display="https://drive.google.com/file/d/17jgZEjslxIZPC5kuzOq6oTK5EuDiJ-_l/view?usp=drive_link"/>
-    <hyperlink ref="F44" r:id="rId12" display="https://drive.google.com/file/d/1miMp-AR_hOfLUWszGb_aZG2f_Nd66Ntt/view?usp=drive_link"/>
-    <hyperlink ref="F50" r:id="rId13" display="https://drive.google.com/file/d/1Skq_uMcAR08LMDnIpOswjxm5ntbVXm5M/view?usp=drive_link"/>
-    <hyperlink ref="F49" r:id="rId14" display="https://drive.google.com/file/d/1mN12zjCiawfU4k1ifPsLW-hcuzPV7Voz/view?usp=drive_link"/>
-    <hyperlink ref="F51" r:id="rId15" display="https://drive.google.com/file/d/1KSYs7ZOhEkjBQX5UnMpLkbxZZ6BLhbDm/view?usp=drive_link"/>
-    <hyperlink ref="F53" r:id="rId16" display="https://drive.google.com/file/d/1geppLqwV80p66bXdffVBbLayjCkIQ9mk/view?usp=drive_link"/>
-    <hyperlink ref="F55" r:id="rId17" display="https://drive.google.com/file/d/1T58G_EIr4pWZYJ8plXEWspFHr35g-Nsy/view?usp=drive_link"/>
-    <hyperlink ref="F6" r:id="rId8" display="https://drive.google.com/drive/folders/18PTnMwgyhxIWTVNLMwf0sbzhvh9AlVqE?usp=drive_link"/>
-    <hyperlink ref="F13" r:id="rId8" display="https://drive.google.com/drive/folders/18PTnMwgyhxIWTVNLMwf0sbzhvh9AlVqE?usp=drive_link"/>
-    <hyperlink ref="F8" r:id="rId18" display="https://drive.google.com/file/d/1M-PAz9S7cvYR8T6-VIEZKMbw7yVTN5je/view?usp=drive_link"/>
-    <hyperlink ref="C12" r:id="rId19" display="https://osworld-grounding.github.io/"/>
-    <hyperlink ref="C16" r:id="rId19" display="https://osworld-grounding.github.io/"/>
-    <hyperlink ref="C18" r:id="rId19" display="https://osworld-grounding.github.io/"/>
-    <hyperlink ref="C21" r:id="rId19" display="https://osworld-grounding.github.io/"/>
-    <hyperlink ref="F14" r:id="rId20" display="https://drive.google.com/file/d/1t-w6OAQHfmRplHbi93aWXZlOBwOQkwY2/view?usp=drive_link"/>
-    <hyperlink ref="C4" r:id="rId21" display="https://help.openai.com/en/articles/10561834-operator-release-notes"/>
-    <hyperlink ref="C32" r:id="rId22" display="https://arxiv.org/abs/2505.13909"/>
-    <hyperlink ref="C10" r:id="rId23" display="https://arxiv.org/abs/2505.16282"/>
-    <hyperlink ref="C23" r:id="rId24" display="https://arxiv.org/abs/2505.23762"/>
-    <hyperlink ref="C8" r:id="rId25" display="https://arxiv.org/abs/2505.10887"/>
-    <hyperlink ref="F3" r:id="rId26" display="https://drive.google.com/drive/folders/1GvNXwDt5_U-ned49urVlOFj1FBi86ddT?usp=sharing"/>
-    <hyperlink ref="C3" r:id="rId27" display="https://arxiv.org/abs/2507.05791"/>
-    <hyperlink ref="C56" r:id="rId28" display="https://arxiv.org/abs/2312.08914"/>
-    <hyperlink ref="C2" r:id="rId29" display="https://www.askui.com/"/>
+    <hyperlink ref="C42" ns1:id="rId1" display="https://arxiv.org/abs/2504.07491"/>
+    <hyperlink ref="C6" ns1:id="rId2" display="https://seed-tars.com/1.5"/>
+    <hyperlink ref="C7" ns1:id="rId3" display="https://github.com/simular-ai/Agent-S"/>
+    <hyperlink ref="C15" ns1:id="rId2" display="https://seed-tars.com/1.5" tooltip="https://seed-tars.com/1.5"/>
+    <hyperlink ref="F6" ns1:id="rId4" display="https://drive.google.com/file/d/1e7SCYqpxFX2FCGEOhf6jcVvwkx3leIKf/view?usp=drive_link"/>
+    <hyperlink ref="F18" ns1:id="rId5" display="https://drive.google.com/file/d/1vUWlXVenkOc5F1s-z8DdpfU4Y5fUMssr/view?usp=drive_link" tooltip="https://drive.google.com/file/d/1vUWlXVenkOc5F1s-z8DdpfU4Y5fUMssr/view?usp=drive_link"/>
+    <hyperlink ref="F44" ns1:id="rId6" display="https://drive.google.com/drive/folders/14_xlL-e0-0INq2O1THbhFKi6Z0bgfwR4?usp=drive_link"/>
+    <hyperlink ref="F48" ns1:id="rId7" display="https://drive.google.com/drive/folders/1j-YVzEGAGWxXgse75MCnhUCTVuejM76A?usp=drive_link"/>
+    <hyperlink ref="F10" ns1:id="rId8" display="https://drive.google.com/drive/folders/18PTnMwgyhxIWTVNLMwf0sbzhvh9AlVqE?usp=drive_link" tooltip="https://drive.google.com/drive/folders/18PTnMwgyhxIWTVNLMwf0sbzhvh9AlVqE?usp=drive_link"/>
+    <hyperlink ref="F47" ns1:id="rId9" display="https://drive.google.com/drive/folders/1NLsHdLUNZOHsEC5xNZ4e4PHkDC5IELjj?usp=drive_link"/>
+    <hyperlink ref="F55" ns1:id="rId10" display="https://drive.google.com/drive/folders/1iBOXZpknCi1Fqzg0fQMG6CZc9NWrwdkf?usp=drive_link"/>
+    <hyperlink ref="F46" ns1:id="rId11" display="https://drive.google.com/file/d/17jgZEjslxIZPC5kuzOq6oTK5EuDiJ-_l/view?usp=drive_link"/>
+    <hyperlink ref="F45" ns1:id="rId12" display="https://drive.google.com/file/d/1miMp-AR_hOfLUWszGb_aZG2f_Nd66Ntt/view?usp=drive_link"/>
+    <hyperlink ref="F51" ns1:id="rId13" display="https://drive.google.com/file/d/1Skq_uMcAR08LMDnIpOswjxm5ntbVXm5M/view?usp=drive_link"/>
+    <hyperlink ref="F50" ns1:id="rId14" display="https://drive.google.com/file/d/1mN12zjCiawfU4k1ifPsLW-hcuzPV7Voz/view?usp=drive_link"/>
+    <hyperlink ref="F52" ns1:id="rId15" display="https://drive.google.com/file/d/1KSYs7ZOhEkjBQX5UnMpLkbxZZ6BLhbDm/view?usp=drive_link"/>
+    <hyperlink ref="F54" ns1:id="rId16" display="https://drive.google.com/file/d/1geppLqwV80p66bXdffVBbLayjCkIQ9mk/view?usp=drive_link"/>
+    <hyperlink ref="F56" ns1:id="rId17" display="https://drive.google.com/file/d/1T58G_EIr4pWZYJ8plXEWspFHr35g-Nsy/view?usp=drive_link"/>
+    <hyperlink ref="F7" ns1:id="rId8" display="https://drive.google.com/drive/folders/18PTnMwgyhxIWTVNLMwf0sbzhvh9AlVqE?usp=drive_link"/>
+    <hyperlink ref="F14" ns1:id="rId8" display="https://drive.google.com/drive/folders/18PTnMwgyhxIWTVNLMwf0sbzhvh9AlVqE?usp=drive_link"/>
+    <hyperlink ref="F9" ns1:id="rId18" display="https://drive.google.com/file/d/1M-PAz9S7cvYR8T6-VIEZKMbw7yVTN5je/view?usp=drive_link"/>
+    <hyperlink ref="C13" ns1:id="rId19" display="https://osworld-grounding.github.io/"/>
+    <hyperlink ref="C17" ns1:id="rId19" display="https://osworld-grounding.github.io/"/>
+    <hyperlink ref="C19" ns1:id="rId19" display="https://osworld-grounding.github.io/"/>
+    <hyperlink ref="C22" ns1:id="rId19" display="https://osworld-grounding.github.io/"/>
+    <hyperlink ref="F15" ns1:id="rId20" display="https://drive.google.com/file/d/1t-w6OAQHfmRplHbi93aWXZlOBwOQkwY2/view?usp=drive_link"/>
+    <hyperlink ref="C5" ns1:id="rId21" display="https://help.openai.com/en/articles/10561834-operator-release-notes"/>
+    <hyperlink ref="C33" ns1:id="rId22" display="https://arxiv.org/abs/2505.13909"/>
+    <hyperlink ref="C11" ns1:id="rId23" display="https://arxiv.org/abs/2505.16282"/>
+    <hyperlink ref="C24" ns1:id="rId24" display="https://arxiv.org/abs/2505.23762"/>
+    <hyperlink ref="C9" ns1:id="rId25" display="https://arxiv.org/abs/2505.10887"/>
+    <hyperlink ref="F4" ns1:id="rId26" display="https://drive.google.com/drive/folders/1GvNXwDt5_U-ned49urVlOFj1FBi86ddT?usp=sharing"/>
+    <hyperlink ref="C4" ns1:id="rId27" display="https://arxiv.org/abs/2507.05791"/>
+    <hyperlink ref="C57" ns1:id="rId28" display="https://arxiv.org/abs/2312.08914"/>
+    <hyperlink ref="C2" ns1:id="rId29" display="https://www.askui.com/"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>